<commit_message>
Begrippen in Excel-sheet alfabetisch gesorteerd.
</commit_message>
<xml_diff>
--- a/excel/2026-06-26 Begrippenkader Beslag (2).xlsx
+++ b/excel/2026-06-26 Begrippenkader Beslag (2).xlsx
@@ -1,21 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Mijn Documenten\GitHub\begrippenkader-beslag\excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB430147-5F49-4C6F-9473-4E3E4CADC9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="432">
   <si>
     <t>Titel</t>
   </si>
@@ -1316,14 +1326,9 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1350,13 +1355,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1646,14 +1659,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AP115"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:42">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1781,9 +1791,9 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:42">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>366</v>
       </c>
       <c r="B2" t="s">
         <v>43</v>
@@ -1792,21 +1802,24 @@
         <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>367</v>
       </c>
       <c r="J2" t="s">
-        <v>46</v>
+        <v>368</v>
+      </c>
+      <c r="W2" t="s">
+        <v>162</v>
       </c>
       <c r="AJ2" t="s">
         <v>47</v>
       </c>
       <c r="AO2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:42">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>159</v>
       </c>
       <c r="B3" t="s">
         <v>43</v>
@@ -1815,21 +1828,24 @@
         <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="J3" t="s">
-        <v>51</v>
+        <v>161</v>
+      </c>
+      <c r="W3" t="s">
+        <v>162</v>
       </c>
       <c r="AJ3" t="s">
         <v>47</v>
       </c>
       <c r="AO3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:42">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
         <v>43</v>
@@ -1838,21 +1854,18 @@
         <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="J4" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="AJ4" t="s">
         <v>47</v>
       </c>
-      <c r="AO4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="5" spans="1:42">
+    </row>
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>353</v>
       </c>
       <c r="B5" t="s">
         <v>43</v>
@@ -1861,10 +1874,10 @@
         <v>44</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>354</v>
       </c>
       <c r="J5" t="s">
-        <v>58</v>
+        <v>355</v>
       </c>
       <c r="AJ5" t="s">
         <v>47</v>
@@ -1873,113 +1886,107 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:42">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" t="s">
+        <v>351</v>
+      </c>
+      <c r="J6" t="s">
+        <v>352</v>
+      </c>
+      <c r="P6" t="s">
+        <v>71</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" t="s">
+        <v>109</v>
+      </c>
+      <c r="J7" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s">
+        <v>78</v>
+      </c>
+      <c r="J8" t="s">
+        <v>79</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>59</v>
       </c>
-      <c r="B6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
         <v>60</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J9" t="s">
         <v>61</v>
       </c>
-      <c r="R6" t="s">
+      <c r="R9" t="s">
         <v>62</v>
       </c>
-      <c r="T6" t="s">
+      <c r="T9" t="s">
         <v>63</v>
       </c>
-      <c r="AJ6" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO6" t="s">
+      <c r="AJ9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO9" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:42">
-      <c r="A7" t="s">
-        <v>65</v>
-      </c>
-      <c r="B7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" t="s">
-        <v>66</v>
-      </c>
-      <c r="J7" t="s">
-        <v>67</v>
-      </c>
-      <c r="L7" t="s">
-        <v>68</v>
-      </c>
-      <c r="S7" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="8" spans="1:42">
-      <c r="A8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AJ8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:42">
-      <c r="A9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" t="s">
-        <v>76</v>
-      </c>
-      <c r="J9" t="s">
-        <v>58</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:42">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>77</v>
+        <v>383</v>
       </c>
       <c r="B10" t="s">
         <v>43</v>
@@ -1988,10 +1995,10 @@
         <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>384</v>
       </c>
       <c r="J10" t="s">
-        <v>79</v>
+        <v>385</v>
       </c>
       <c r="AJ10" t="s">
         <v>47</v>
@@ -2000,9 +2007,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:42">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
         <v>43</v>
@@ -2011,364 +2018,391 @@
         <v>44</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="J11" t="s">
-        <v>82</v>
+        <v>95</v>
+      </c>
+      <c r="L11" t="s">
+        <v>96</v>
       </c>
       <c r="AJ11" t="s">
         <v>47</v>
       </c>
       <c r="AO11" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>228</v>
+      </c>
+      <c r="J12" t="s">
+        <v>229</v>
+      </c>
+      <c r="L12" t="s">
+        <v>104</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>162</v>
+      </c>
+      <c r="B13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>363</v>
+      </c>
+      <c r="J13" t="s">
+        <v>364</v>
+      </c>
+      <c r="L13" t="s">
+        <v>104</v>
+      </c>
+      <c r="R13" t="s">
+        <v>59</v>
+      </c>
+      <c r="X13" t="s">
+        <v>365</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>419</v>
+      </c>
+      <c r="B14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s">
+        <v>420</v>
+      </c>
+      <c r="J14" t="s">
+        <v>421</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>145</v>
+      </c>
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s">
+        <v>146</v>
+      </c>
+      <c r="J15" t="s">
+        <v>147</v>
+      </c>
+      <c r="W15" t="s">
+        <v>148</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s">
+        <v>130</v>
+      </c>
+      <c r="E16" t="s">
+        <v>131</v>
+      </c>
+      <c r="J16" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>133</v>
+      </c>
+      <c r="R16" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s">
+        <v>153</v>
+      </c>
+      <c r="E17" t="s">
+        <v>154</v>
+      </c>
+      <c r="J17" t="s">
+        <v>155</v>
+      </c>
+      <c r="M17" t="s">
+        <v>104</v>
+      </c>
+      <c r="R17" t="s">
+        <v>156</v>
+      </c>
+      <c r="X17" t="s">
+        <v>157</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>395</v>
+      </c>
+      <c r="B18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>396</v>
+      </c>
+      <c r="J18" t="s">
+        <v>397</v>
+      </c>
+      <c r="AJ18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO18" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="1:42">
-      <c r="A12" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" t="s">
-        <v>84</v>
-      </c>
-      <c r="J12" t="s">
-        <v>85</v>
-      </c>
-      <c r="P12" t="s">
-        <v>86</v>
-      </c>
-      <c r="R12" t="s">
-        <v>87</v>
-      </c>
-      <c r="AJ12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:42">
-      <c r="A13" t="s">
-        <v>88</v>
-      </c>
-      <c r="B13" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" t="s">
-        <v>89</v>
-      </c>
-      <c r="J13" t="s">
-        <v>90</v>
-      </c>
-      <c r="R13" t="s">
+    <row r="19" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
+        <v>193</v>
+      </c>
+      <c r="J19" t="s">
+        <v>194</v>
+      </c>
+      <c r="R19" t="s">
+        <v>195</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>148</v>
+      </c>
+      <c r="B20" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>167</v>
+      </c>
+      <c r="J20" t="s">
+        <v>168</v>
+      </c>
+      <c r="L20" t="s">
+        <v>169</v>
+      </c>
+      <c r="X20" t="s">
+        <v>170</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>379</v>
+      </c>
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
+        <v>380</v>
+      </c>
+      <c r="J21" t="s">
+        <v>381</v>
+      </c>
+      <c r="AJ21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="22" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>426</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
+        <v>427</v>
+      </c>
+      <c r="J22" t="s">
+        <v>428</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="23" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>238</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s">
+        <v>239</v>
+      </c>
+      <c r="E23" t="s">
+        <v>240</v>
+      </c>
+      <c r="J23" t="s">
+        <v>241</v>
+      </c>
+      <c r="L23" t="s">
+        <v>242</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>401</v>
+      </c>
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>402</v>
+      </c>
+      <c r="J24" t="s">
+        <v>403</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>315</v>
+      </c>
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s">
+        <v>316</v>
+      </c>
+      <c r="E25" t="s">
+        <v>317</v>
+      </c>
+      <c r="J25" t="s">
+        <v>318</v>
+      </c>
+      <c r="W25" t="s">
         <v>91</v>
       </c>
-      <c r="AJ13" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="14" spans="1:42">
-      <c r="A14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B14" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" t="s">
-        <v>94</v>
-      </c>
-      <c r="J14" t="s">
-        <v>95</v>
-      </c>
-      <c r="L14" t="s">
-        <v>96</v>
-      </c>
-      <c r="AJ14" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO14" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:42">
-      <c r="A15" t="s">
-        <v>98</v>
-      </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" t="s">
-        <v>99</v>
-      </c>
-      <c r="J15" t="s">
-        <v>100</v>
-      </c>
-      <c r="AJ15" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO15" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="16" spans="1:42">
-      <c r="A16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B16" t="s">
-        <v>43</v>
-      </c>
-      <c r="C16" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" t="s">
-        <v>102</v>
-      </c>
-      <c r="J16" t="s">
-        <v>103</v>
-      </c>
-      <c r="L16" t="s">
-        <v>104</v>
-      </c>
-      <c r="AJ16" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO16" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" spans="1:42">
-      <c r="A17" t="s">
-        <v>105</v>
-      </c>
-      <c r="B17" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" t="s">
-        <v>106</v>
-      </c>
-      <c r="J17" t="s">
-        <v>107</v>
-      </c>
-      <c r="AJ17" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="18" spans="1:42">
-      <c r="A18" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" t="s">
-        <v>109</v>
-      </c>
-      <c r="J18" t="s">
-        <v>110</v>
-      </c>
-      <c r="AJ18" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:42">
-      <c r="A19" t="s">
-        <v>111</v>
-      </c>
-      <c r="B19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19" t="s">
-        <v>112</v>
-      </c>
-      <c r="J19" t="s">
-        <v>113</v>
-      </c>
-      <c r="AJ19" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO19" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:42">
-      <c r="A20" t="s">
-        <v>114</v>
-      </c>
-      <c r="B20" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" t="s">
-        <v>115</v>
-      </c>
-      <c r="J20" t="s">
-        <v>116</v>
-      </c>
-      <c r="AJ20" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO20" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:42">
-      <c r="A21" t="s">
-        <v>117</v>
-      </c>
-      <c r="B21" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" t="s">
-        <v>44</v>
-      </c>
-      <c r="D21" t="s">
-        <v>118</v>
-      </c>
-      <c r="J21" t="s">
-        <v>119</v>
-      </c>
-      <c r="AJ21" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO21" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:42">
-      <c r="A22" t="s">
-        <v>120</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" t="s">
-        <v>121</v>
-      </c>
-      <c r="J22" t="s">
-        <v>122</v>
-      </c>
-      <c r="W22" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ22" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO22" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="23" spans="1:42">
-      <c r="A23" t="s">
-        <v>123</v>
-      </c>
-      <c r="B23" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" t="s">
-        <v>124</v>
-      </c>
-      <c r="J23" t="s">
-        <v>125</v>
-      </c>
-      <c r="AJ23" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO23" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="24" spans="1:42">
-      <c r="A24" t="s">
-        <v>126</v>
-      </c>
-      <c r="B24" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" t="s">
-        <v>127</v>
-      </c>
-      <c r="J24" t="s">
-        <v>128</v>
-      </c>
-      <c r="S24" t="s">
-        <v>129</v>
-      </c>
-      <c r="AJ24" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO24" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:42">
-      <c r="A25" t="s">
-        <v>86</v>
-      </c>
-      <c r="B25" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" t="s">
-        <v>130</v>
-      </c>
-      <c r="E25" t="s">
-        <v>131</v>
-      </c>
-      <c r="J25" t="s">
-        <v>132</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>133</v>
-      </c>
-      <c r="R25" t="s">
-        <v>59</v>
-      </c>
       <c r="AJ25" t="s">
         <v>47</v>
       </c>
       <c r="AO25" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:42">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="26" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>134</v>
+        <v>289</v>
       </c>
       <c r="B26" t="s">
         <v>43</v>
@@ -2377,10 +2411,10 @@
         <v>44</v>
       </c>
       <c r="D26" t="s">
-        <v>135</v>
+        <v>290</v>
       </c>
       <c r="J26" t="s">
-        <v>136</v>
+        <v>291</v>
       </c>
       <c r="AJ26" t="s">
         <v>47</v>
@@ -2389,9 +2423,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:42">
+    <row r="27" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>137</v>
+        <v>184</v>
       </c>
       <c r="B27" t="s">
         <v>43</v>
@@ -2400,212 +2434,209 @@
         <v>44</v>
       </c>
       <c r="D27" t="s">
-        <v>138</v>
+        <v>185</v>
       </c>
       <c r="J27" t="s">
-        <v>139</v>
-      </c>
-      <c r="R27" t="s">
-        <v>140</v>
-      </c>
-      <c r="S27" t="s">
+        <v>186</v>
+      </c>
+      <c r="L27" t="s">
+        <v>187</v>
+      </c>
+      <c r="AJ27" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO27" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>215</v>
+      </c>
+      <c r="B28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s">
+        <v>216</v>
+      </c>
+      <c r="J28" t="s">
+        <v>217</v>
+      </c>
+      <c r="R28" t="s">
+        <v>218</v>
+      </c>
+      <c r="S28" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ28" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO28" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>87</v>
+      </c>
+      <c r="B29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" t="s">
+        <v>236</v>
+      </c>
+      <c r="J29" t="s">
+        <v>237</v>
+      </c>
+      <c r="P29" t="s">
+        <v>86</v>
+      </c>
+      <c r="R29" t="s">
+        <v>83</v>
+      </c>
+      <c r="AJ29" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>376</v>
+      </c>
+      <c r="B30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" t="s">
+        <v>377</v>
+      </c>
+      <c r="J30" t="s">
+        <v>378</v>
+      </c>
+      <c r="AJ30" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO30" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" t="s">
+        <v>66</v>
+      </c>
+      <c r="J31" t="s">
+        <v>67</v>
+      </c>
+      <c r="L31" t="s">
+        <v>68</v>
+      </c>
+      <c r="S31" t="s">
         <v>69</v>
       </c>
-      <c r="AJ27" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO27" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="28" spans="1:42">
-      <c r="A28" t="s">
-        <v>142</v>
-      </c>
-      <c r="B28" t="s">
-        <v>43</v>
-      </c>
-      <c r="C28" t="s">
-        <v>44</v>
-      </c>
-      <c r="D28" t="s">
-        <v>143</v>
-      </c>
-      <c r="J28" t="s">
-        <v>144</v>
-      </c>
-      <c r="AJ28" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO28" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:42">
-      <c r="A29" t="s">
-        <v>145</v>
-      </c>
-      <c r="B29" t="s">
-        <v>43</v>
-      </c>
-      <c r="C29" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" t="s">
-        <v>146</v>
-      </c>
-      <c r="J29" t="s">
-        <v>147</v>
-      </c>
-      <c r="W29" t="s">
+      <c r="AJ31" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>274</v>
+      </c>
+      <c r="B32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
+        <v>275</v>
+      </c>
+      <c r="J32" t="s">
+        <v>276</v>
+      </c>
+      <c r="W32" t="s">
         <v>148</v>
       </c>
-      <c r="AJ29" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO29" t="s">
+      <c r="AJ32" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO32" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="33" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>303</v>
+      </c>
+      <c r="B33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" t="s">
+        <v>304</v>
+      </c>
+      <c r="J33" t="s">
+        <v>305</v>
+      </c>
+      <c r="S33" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ33" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>295</v>
+      </c>
+      <c r="B34" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" t="s">
+        <v>371</v>
+      </c>
+      <c r="J34" t="s">
+        <v>372</v>
+      </c>
+      <c r="P34" t="s">
+        <v>292</v>
+      </c>
+      <c r="AJ34" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO34" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="1:42">
-      <c r="A30" t="s">
-        <v>149</v>
-      </c>
-      <c r="B30" t="s">
-        <v>43</v>
-      </c>
-      <c r="C30" t="s">
-        <v>44</v>
-      </c>
-      <c r="D30" t="s">
-        <v>150</v>
-      </c>
-      <c r="J30" t="s">
-        <v>151</v>
-      </c>
-      <c r="L30" t="s">
-        <v>152</v>
-      </c>
-      <c r="AJ30" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO30" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="31" spans="1:42">
-      <c r="A31" t="s">
-        <v>91</v>
-      </c>
-      <c r="B31" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31" t="s">
-        <v>153</v>
-      </c>
-      <c r="E31" t="s">
-        <v>154</v>
-      </c>
-      <c r="J31" t="s">
-        <v>155</v>
-      </c>
-      <c r="M31" t="s">
-        <v>104</v>
-      </c>
-      <c r="R31" t="s">
-        <v>156</v>
-      </c>
-      <c r="X31" t="s">
-        <v>157</v>
-      </c>
-      <c r="AJ31" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO31" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="32" spans="1:42">
-      <c r="A32" t="s">
-        <v>159</v>
-      </c>
-      <c r="B32" t="s">
-        <v>43</v>
-      </c>
-      <c r="C32" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" t="s">
-        <v>160</v>
-      </c>
-      <c r="J32" t="s">
-        <v>161</v>
-      </c>
-      <c r="W32" t="s">
-        <v>162</v>
-      </c>
-      <c r="AJ32" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO32" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="33" spans="1:42">
-      <c r="A33" t="s">
-        <v>164</v>
-      </c>
-      <c r="B33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" t="s">
-        <v>165</v>
-      </c>
-      <c r="J33" t="s">
-        <v>166</v>
-      </c>
-      <c r="AJ33" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="1:42">
-      <c r="A34" t="s">
-        <v>148</v>
-      </c>
-      <c r="B34" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" t="s">
-        <v>167</v>
-      </c>
-      <c r="J34" t="s">
-        <v>168</v>
-      </c>
-      <c r="L34" t="s">
-        <v>169</v>
-      </c>
-      <c r="X34" t="s">
-        <v>170</v>
-      </c>
-      <c r="AJ34" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="35" spans="1:42">
+    <row r="35" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>171</v>
+        <v>262</v>
       </c>
       <c r="B35" t="s">
         <v>43</v>
@@ -2614,16 +2645,10 @@
         <v>44</v>
       </c>
       <c r="D35" t="s">
-        <v>172</v>
+        <v>263</v>
       </c>
       <c r="J35" t="s">
-        <v>173</v>
-      </c>
-      <c r="R35" t="s">
-        <v>174</v>
-      </c>
-      <c r="W35" t="s">
-        <v>91</v>
+        <v>264</v>
       </c>
       <c r="AJ35" t="s">
         <v>47</v>
@@ -2632,9 +2657,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="36" spans="1:42">
+    <row r="36" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>175</v>
+        <v>252</v>
       </c>
       <c r="B36" t="s">
         <v>43</v>
@@ -2643,21 +2668,24 @@
         <v>44</v>
       </c>
       <c r="D36" t="s">
-        <v>176</v>
+        <v>253</v>
       </c>
       <c r="J36" t="s">
-        <v>177</v>
+        <v>254</v>
+      </c>
+      <c r="L36" t="s">
+        <v>255</v>
+      </c>
+      <c r="R36" t="s">
+        <v>69</v>
       </c>
       <c r="AJ36" t="s">
         <v>47</v>
       </c>
-      <c r="AO36" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="37" spans="1:42">
+    </row>
+    <row r="37" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>178</v>
+        <v>334</v>
       </c>
       <c r="B37" t="s">
         <v>43</v>
@@ -2666,10 +2694,10 @@
         <v>44</v>
       </c>
       <c r="D37" t="s">
-        <v>179</v>
+        <v>335</v>
       </c>
       <c r="J37" t="s">
-        <v>180</v>
+        <v>336</v>
       </c>
       <c r="W37" t="s">
         <v>91</v>
@@ -2678,12 +2706,12 @@
         <v>47</v>
       </c>
       <c r="AO37" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="38" spans="1:42">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="38" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>181</v>
+        <v>283</v>
       </c>
       <c r="B38" t="s">
         <v>43</v>
@@ -2692,21 +2720,18 @@
         <v>44</v>
       </c>
       <c r="D38" t="s">
-        <v>182</v>
+        <v>284</v>
       </c>
       <c r="J38" t="s">
-        <v>183</v>
-      </c>
-      <c r="P38" t="s">
-        <v>129</v>
+        <v>285</v>
       </c>
       <c r="AJ38" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:42">
+    <row r="39" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>184</v>
+        <v>248</v>
       </c>
       <c r="B39" t="s">
         <v>43</v>
@@ -2715,13 +2740,13 @@
         <v>44</v>
       </c>
       <c r="D39" t="s">
-        <v>185</v>
+        <v>249</v>
+      </c>
+      <c r="E39" t="s">
+        <v>250</v>
       </c>
       <c r="J39" t="s">
-        <v>186</v>
-      </c>
-      <c r="L39" t="s">
-        <v>187</v>
+        <v>251</v>
       </c>
       <c r="AJ39" t="s">
         <v>47</v>
@@ -2730,9 +2755,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="40" spans="1:42">
+    <row r="40" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
       <c r="B40" t="s">
         <v>43</v>
@@ -2741,24 +2766,21 @@
         <v>44</v>
       </c>
       <c r="D40" t="s">
-        <v>189</v>
-      </c>
-      <c r="E40" t="s">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="J40" t="s">
-        <v>191</v>
-      </c>
-      <c r="R40" t="s">
-        <v>69</v>
+        <v>166</v>
       </c>
       <c r="AJ40" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="41" spans="1:42">
+      <c r="AO40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>192</v>
+        <v>218</v>
       </c>
       <c r="B41" t="s">
         <v>43</v>
@@ -2767,21 +2789,27 @@
         <v>44</v>
       </c>
       <c r="D41" t="s">
-        <v>193</v>
+        <v>246</v>
       </c>
       <c r="J41" t="s">
-        <v>194</v>
+        <v>247</v>
       </c>
       <c r="R41" t="s">
-        <v>195</v>
+        <v>215</v>
+      </c>
+      <c r="S41" t="s">
+        <v>59</v>
       </c>
       <c r="AJ41" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="42" spans="1:42">
+      <c r="AO41" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="42" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>196</v>
+        <v>323</v>
       </c>
       <c r="B42" t="s">
         <v>43</v>
@@ -2790,24 +2818,27 @@
         <v>44</v>
       </c>
       <c r="D42" t="s">
-        <v>197</v>
+        <v>324</v>
+      </c>
+      <c r="F42" t="s">
+        <v>325</v>
       </c>
       <c r="J42" t="s">
-        <v>198</v>
-      </c>
-      <c r="S42" t="s">
-        <v>129</v>
+        <v>326</v>
+      </c>
+      <c r="L42" t="s">
+        <v>327</v>
       </c>
       <c r="AJ42" t="s">
         <v>47</v>
       </c>
       <c r="AO42" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="43" spans="1:42">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="43" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>200</v>
+        <v>392</v>
       </c>
       <c r="B43" t="s">
         <v>43</v>
@@ -2816,145 +2847,130 @@
         <v>44</v>
       </c>
       <c r="D43" t="s">
-        <v>201</v>
+        <v>393</v>
       </c>
       <c r="J43" t="s">
-        <v>202</v>
+        <v>394</v>
       </c>
       <c r="AJ43" t="s">
         <v>47</v>
       </c>
       <c r="AO43" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="44" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>309</v>
+      </c>
+      <c r="B44" t="s">
+        <v>43</v>
+      </c>
+      <c r="C44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
+        <v>310</v>
+      </c>
+      <c r="J44" t="s">
+        <v>311</v>
+      </c>
+      <c r="AJ44" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>243</v>
+      </c>
+      <c r="B45" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
+        <v>244</v>
+      </c>
+      <c r="J45" t="s">
+        <v>245</v>
+      </c>
+      <c r="AJ45" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO45" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="44" spans="1:42">
-      <c r="A44" t="s">
-        <v>203</v>
-      </c>
-      <c r="B44" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" t="s">
-        <v>44</v>
-      </c>
-      <c r="D44" t="s">
-        <v>204</v>
-      </c>
-      <c r="J44" t="s">
-        <v>205</v>
-      </c>
-      <c r="AJ44" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO44" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="45" spans="1:42">
-      <c r="A45" t="s">
-        <v>206</v>
-      </c>
-      <c r="B45" t="s">
-        <v>43</v>
-      </c>
-      <c r="C45" t="s">
-        <v>44</v>
-      </c>
-      <c r="D45" t="s">
-        <v>207</v>
-      </c>
-      <c r="J45" t="s">
-        <v>208</v>
-      </c>
-      <c r="W45" t="s">
-        <v>148</v>
-      </c>
-      <c r="AJ45" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO45" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="46" spans="1:42">
+    <row r="46" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>286</v>
+      </c>
+      <c r="B46" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
+        <v>287</v>
+      </c>
+      <c r="J46" t="s">
+        <v>288</v>
+      </c>
+      <c r="AJ46" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO46" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="47" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>297</v>
+      </c>
+      <c r="B47" t="s">
+        <v>43</v>
+      </c>
+      <c r="C47" t="s">
+        <v>44</v>
+      </c>
+      <c r="D47" t="s">
+        <v>298</v>
+      </c>
+      <c r="J47" t="s">
+        <v>299</v>
+      </c>
+      <c r="AJ47" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO47" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="48" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>209</v>
       </c>
-      <c r="B46" t="s">
-        <v>43</v>
-      </c>
-      <c r="C46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="B48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D48" t="s">
         <v>210</v>
       </c>
-      <c r="J46" t="s">
+      <c r="J48" t="s">
         <v>211</v>
       </c>
-      <c r="AJ46" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="47" spans="1:42">
-      <c r="A47" t="s">
-        <v>129</v>
-      </c>
-      <c r="B47" t="s">
-        <v>43</v>
-      </c>
-      <c r="C47" t="s">
-        <v>44</v>
-      </c>
-      <c r="D47" t="s">
-        <v>212</v>
-      </c>
-      <c r="J47" t="s">
-        <v>213</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>181</v>
-      </c>
-      <c r="T47" t="s">
-        <v>214</v>
-      </c>
-      <c r="AJ47" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="48" spans="1:42">
-      <c r="A48" t="s">
-        <v>215</v>
-      </c>
-      <c r="B48" t="s">
-        <v>43</v>
-      </c>
-      <c r="C48" t="s">
-        <v>44</v>
-      </c>
-      <c r="D48" t="s">
-        <v>216</v>
-      </c>
-      <c r="J48" t="s">
-        <v>217</v>
-      </c>
-      <c r="R48" t="s">
-        <v>218</v>
-      </c>
-      <c r="S48" t="s">
-        <v>59</v>
-      </c>
       <c r="AJ48" t="s">
         <v>47</v>
       </c>
-      <c r="AO48" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="49" spans="1:42">
+    </row>
+    <row r="49" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>219</v>
+        <v>83</v>
       </c>
       <c r="B49" t="s">
         <v>43</v>
@@ -2963,24 +2979,24 @@
         <v>44</v>
       </c>
       <c r="D49" t="s">
-        <v>220</v>
+        <v>84</v>
       </c>
       <c r="J49" t="s">
-        <v>221</v>
-      </c>
-      <c r="S49" t="s">
-        <v>222</v>
+        <v>85</v>
+      </c>
+      <c r="P49" t="s">
+        <v>86</v>
+      </c>
+      <c r="R49" t="s">
+        <v>87</v>
       </c>
       <c r="AJ49" t="s">
         <v>47</v>
       </c>
-      <c r="AO49" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="50" spans="1:42">
+    </row>
+    <row r="50" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>224</v>
+        <v>71</v>
       </c>
       <c r="B50" t="s">
         <v>43</v>
@@ -2989,21 +3005,21 @@
         <v>44</v>
       </c>
       <c r="D50" t="s">
-        <v>225</v>
+        <v>72</v>
       </c>
       <c r="J50" t="s">
-        <v>226</v>
+        <v>73</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>74</v>
       </c>
       <c r="AJ50" t="s">
         <v>47</v>
       </c>
-      <c r="AO50" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="51" spans="1:42">
+    </row>
+    <row r="51" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>227</v>
+        <v>259</v>
       </c>
       <c r="B51" t="s">
         <v>43</v>
@@ -3012,13 +3028,10 @@
         <v>44</v>
       </c>
       <c r="D51" t="s">
-        <v>228</v>
+        <v>260</v>
       </c>
       <c r="J51" t="s">
-        <v>229</v>
-      </c>
-      <c r="L51" t="s">
-        <v>104</v>
+        <v>261</v>
       </c>
       <c r="AJ51" t="s">
         <v>47</v>
@@ -3027,9 +3040,9 @@
         <v>55</v>
       </c>
     </row>
-    <row r="52" spans="1:42">
+    <row r="52" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>230</v>
+        <v>359</v>
       </c>
       <c r="B52" t="s">
         <v>43</v>
@@ -3038,21 +3051,24 @@
         <v>44</v>
       </c>
       <c r="D52" t="s">
-        <v>231</v>
+        <v>360</v>
+      </c>
+      <c r="G52" t="s">
+        <v>361</v>
       </c>
       <c r="J52" t="s">
-        <v>232</v>
+        <v>362</v>
+      </c>
+      <c r="S52" t="s">
+        <v>292</v>
       </c>
       <c r="AJ52" t="s">
         <v>47</v>
       </c>
-      <c r="AO52" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="53" spans="1:42">
+    </row>
+    <row r="53" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>233</v>
+        <v>137</v>
       </c>
       <c r="B53" t="s">
         <v>43</v>
@@ -3061,21 +3077,27 @@
         <v>44</v>
       </c>
       <c r="D53" t="s">
-        <v>234</v>
+        <v>138</v>
       </c>
       <c r="J53" t="s">
-        <v>235</v>
+        <v>139</v>
       </c>
       <c r="R53" t="s">
-        <v>192</v>
+        <v>140</v>
+      </c>
+      <c r="S53" t="s">
+        <v>69</v>
       </c>
       <c r="AJ53" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="54" spans="1:42">
+      <c r="AO53" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="54" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>87</v>
+        <v>407</v>
       </c>
       <c r="B54" t="s">
         <v>43</v>
@@ -3084,24 +3106,21 @@
         <v>44</v>
       </c>
       <c r="D54" t="s">
-        <v>236</v>
+        <v>408</v>
       </c>
       <c r="J54" t="s">
-        <v>237</v>
-      </c>
-      <c r="P54" t="s">
-        <v>86</v>
-      </c>
-      <c r="R54" t="s">
-        <v>83</v>
+        <v>409</v>
       </c>
       <c r="AJ54" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="55" spans="1:42">
+      <c r="AO54" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="55" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>238</v>
+        <v>423</v>
       </c>
       <c r="B55" t="s">
         <v>43</v>
@@ -3110,27 +3129,18 @@
         <v>44</v>
       </c>
       <c r="D55" t="s">
-        <v>239</v>
-      </c>
-      <c r="E55" t="s">
-        <v>240</v>
+        <v>424</v>
       </c>
       <c r="J55" t="s">
-        <v>241</v>
-      </c>
-      <c r="L55" t="s">
-        <v>242</v>
-      </c>
-      <c r="AJ55" t="s">
-        <v>47</v>
+        <v>425</v>
       </c>
       <c r="AO55" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="56" spans="1:42">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="56" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>243</v>
+        <v>42</v>
       </c>
       <c r="B56" t="s">
         <v>43</v>
@@ -3139,10 +3149,10 @@
         <v>44</v>
       </c>
       <c r="D56" t="s">
-        <v>244</v>
+        <v>45</v>
       </c>
       <c r="J56" t="s">
-        <v>245</v>
+        <v>46</v>
       </c>
       <c r="AJ56" t="s">
         <v>47</v>
@@ -3151,9 +3161,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="57" spans="1:42">
+    <row r="57" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>218</v>
+        <v>98</v>
       </c>
       <c r="B57" t="s">
         <v>43</v>
@@ -3162,27 +3172,21 @@
         <v>44</v>
       </c>
       <c r="D57" t="s">
-        <v>246</v>
+        <v>99</v>
       </c>
       <c r="J57" t="s">
-        <v>247</v>
-      </c>
-      <c r="R57" t="s">
-        <v>215</v>
-      </c>
-      <c r="S57" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="AJ57" t="s">
         <v>47</v>
       </c>
       <c r="AO57" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="58" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>248</v>
+        <v>271</v>
       </c>
       <c r="B58" t="s">
         <v>43</v>
@@ -3191,24 +3195,21 @@
         <v>44</v>
       </c>
       <c r="D58" t="s">
-        <v>249</v>
-      </c>
-      <c r="E58" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="J58" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="AJ58" t="s">
         <v>47</v>
       </c>
       <c r="AO58" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="59" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="59" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>252</v>
+        <v>429</v>
       </c>
       <c r="B59" t="s">
         <v>43</v>
@@ -3217,24 +3218,18 @@
         <v>44</v>
       </c>
       <c r="D59" t="s">
-        <v>253</v>
+        <v>430</v>
       </c>
       <c r="J59" t="s">
-        <v>254</v>
-      </c>
-      <c r="L59" t="s">
-        <v>255</v>
-      </c>
-      <c r="R59" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ59" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="60" spans="1:42">
+        <v>431</v>
+      </c>
+      <c r="AO59" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="60" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>256</v>
+        <v>386</v>
       </c>
       <c r="B60" t="s">
         <v>43</v>
@@ -3243,10 +3238,10 @@
         <v>44</v>
       </c>
       <c r="D60" t="s">
-        <v>257</v>
+        <v>387</v>
       </c>
       <c r="J60" t="s">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="AJ60" t="s">
         <v>47</v>
@@ -3255,9 +3250,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="61" spans="1:42">
+    <row r="61" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>259</v>
+        <v>196</v>
       </c>
       <c r="B61" t="s">
         <v>43</v>
@@ -3266,21 +3261,24 @@
         <v>44</v>
       </c>
       <c r="D61" t="s">
-        <v>260</v>
+        <v>197</v>
       </c>
       <c r="J61" t="s">
-        <v>261</v>
+        <v>198</v>
+      </c>
+      <c r="S61" t="s">
+        <v>129</v>
       </c>
       <c r="AJ61" t="s">
         <v>47</v>
       </c>
       <c r="AO61" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="62" spans="1:42">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="62" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>262</v>
+        <v>219</v>
       </c>
       <c r="B62" t="s">
         <v>43</v>
@@ -3289,67 +3287,70 @@
         <v>44</v>
       </c>
       <c r="D62" t="s">
-        <v>263</v>
+        <v>220</v>
       </c>
       <c r="J62" t="s">
-        <v>264</v>
+        <v>221</v>
+      </c>
+      <c r="S62" t="s">
+        <v>222</v>
       </c>
       <c r="AJ62" t="s">
         <v>47</v>
       </c>
       <c r="AO62" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="63" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>230</v>
+      </c>
+      <c r="B63" t="s">
+        <v>43</v>
+      </c>
+      <c r="C63" t="s">
+        <v>44</v>
+      </c>
+      <c r="D63" t="s">
+        <v>231</v>
+      </c>
+      <c r="J63" t="s">
+        <v>232</v>
+      </c>
+      <c r="AJ63" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO63" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="64" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>114</v>
+      </c>
+      <c r="B64" t="s">
+        <v>43</v>
+      </c>
+      <c r="C64" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64" t="s">
+        <v>115</v>
+      </c>
+      <c r="J64" t="s">
+        <v>116</v>
+      </c>
+      <c r="AJ64" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO64" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="63" spans="1:42">
-      <c r="A63" t="s">
-        <v>265</v>
-      </c>
-      <c r="B63" t="s">
-        <v>43</v>
-      </c>
-      <c r="C63" t="s">
-        <v>44</v>
-      </c>
-      <c r="D63" t="s">
-        <v>266</v>
-      </c>
-      <c r="J63" t="s">
-        <v>267</v>
-      </c>
-      <c r="AJ63" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO63" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="64" spans="1:42">
-      <c r="A64" t="s">
-        <v>268</v>
-      </c>
-      <c r="B64" t="s">
-        <v>43</v>
-      </c>
-      <c r="C64" t="s">
-        <v>44</v>
-      </c>
-      <c r="D64" t="s">
-        <v>269</v>
-      </c>
-      <c r="J64" t="s">
-        <v>270</v>
-      </c>
-      <c r="S64" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ64" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="65" spans="1:42">
+    <row r="65" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>271</v>
+        <v>356</v>
       </c>
       <c r="B65" t="s">
         <v>43</v>
@@ -3358,10 +3359,10 @@
         <v>44</v>
       </c>
       <c r="D65" t="s">
-        <v>272</v>
+        <v>357</v>
       </c>
       <c r="J65" t="s">
-        <v>273</v>
+        <v>358</v>
       </c>
       <c r="AJ65" t="s">
         <v>47</v>
@@ -3370,9 +3371,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="66" spans="1:42">
+    <row r="66" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>274</v>
+        <v>224</v>
       </c>
       <c r="B66" t="s">
         <v>43</v>
@@ -3381,185 +3382,194 @@
         <v>44</v>
       </c>
       <c r="D66" t="s">
-        <v>275</v>
+        <v>225</v>
       </c>
       <c r="J66" t="s">
-        <v>276</v>
-      </c>
-      <c r="W66" t="s">
+        <v>226</v>
+      </c>
+      <c r="AJ66" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO66" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="67" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>306</v>
+      </c>
+      <c r="B67" t="s">
+        <v>43</v>
+      </c>
+      <c r="C67" t="s">
+        <v>44</v>
+      </c>
+      <c r="D67" t="s">
+        <v>307</v>
+      </c>
+      <c r="J67" t="s">
+        <v>308</v>
+      </c>
+      <c r="AJ67" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO67" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>292</v>
+      </c>
+      <c r="B68" t="s">
+        <v>43</v>
+      </c>
+      <c r="C68" t="s">
+        <v>44</v>
+      </c>
+      <c r="D68" t="s">
+        <v>293</v>
+      </c>
+      <c r="J68" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>295</v>
+      </c>
+      <c r="T68" t="s">
+        <v>296</v>
+      </c>
+      <c r="AJ68" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="69" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>134</v>
+      </c>
+      <c r="B69" t="s">
+        <v>43</v>
+      </c>
+      <c r="C69" t="s">
+        <v>44</v>
+      </c>
+      <c r="D69" t="s">
+        <v>135</v>
+      </c>
+      <c r="J69" t="s">
+        <v>136</v>
+      </c>
+      <c r="AJ69" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO69" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="70" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>233</v>
+      </c>
+      <c r="B70" t="s">
+        <v>43</v>
+      </c>
+      <c r="C70" t="s">
+        <v>44</v>
+      </c>
+      <c r="D70" t="s">
+        <v>234</v>
+      </c>
+      <c r="J70" t="s">
+        <v>235</v>
+      </c>
+      <c r="R70" t="s">
+        <v>192</v>
+      </c>
+      <c r="AJ70" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="71" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>206</v>
+      </c>
+      <c r="B71" t="s">
+        <v>43</v>
+      </c>
+      <c r="C71" t="s">
+        <v>44</v>
+      </c>
+      <c r="D71" t="s">
+        <v>207</v>
+      </c>
+      <c r="J71" t="s">
+        <v>208</v>
+      </c>
+      <c r="W71" t="s">
         <v>148</v>
       </c>
-      <c r="AJ66" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO66" t="s">
+      <c r="AJ71" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO71" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="72" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>222</v>
+      </c>
+      <c r="B72" t="s">
+        <v>43</v>
+      </c>
+      <c r="C72" t="s">
+        <v>44</v>
+      </c>
+      <c r="D72" t="s">
+        <v>348</v>
+      </c>
+      <c r="J72" t="s">
+        <v>349</v>
+      </c>
+      <c r="S72" t="s">
+        <v>292</v>
+      </c>
+      <c r="T72" t="s">
+        <v>350</v>
+      </c>
+      <c r="AJ72" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="73" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>126</v>
+      </c>
+      <c r="B73" t="s">
+        <v>43</v>
+      </c>
+      <c r="C73" t="s">
+        <v>44</v>
+      </c>
+      <c r="D73" t="s">
+        <v>127</v>
+      </c>
+      <c r="J73" t="s">
+        <v>128</v>
+      </c>
+      <c r="S73" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ73" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO73" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="67" spans="1:42">
-      <c r="A67" t="s">
-        <v>277</v>
-      </c>
-      <c r="B67" t="s">
-        <v>43</v>
-      </c>
-      <c r="C67" t="s">
-        <v>44</v>
-      </c>
-      <c r="D67" t="s">
-        <v>278</v>
-      </c>
-      <c r="J67" t="s">
-        <v>279</v>
-      </c>
-      <c r="AJ67" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO67" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="68" spans="1:42">
-      <c r="A68" t="s">
-        <v>280</v>
-      </c>
-      <c r="B68" t="s">
-        <v>43</v>
-      </c>
-      <c r="C68" t="s">
-        <v>44</v>
-      </c>
-      <c r="D68" t="s">
-        <v>281</v>
-      </c>
-      <c r="J68" t="s">
-        <v>282</v>
-      </c>
-      <c r="AJ68" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO68" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="69" spans="1:42">
-      <c r="A69" t="s">
-        <v>283</v>
-      </c>
-      <c r="B69" t="s">
-        <v>43</v>
-      </c>
-      <c r="C69" t="s">
-        <v>44</v>
-      </c>
-      <c r="D69" t="s">
-        <v>284</v>
-      </c>
-      <c r="J69" t="s">
-        <v>285</v>
-      </c>
-      <c r="AJ69" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="70" spans="1:42">
-      <c r="A70" t="s">
-        <v>286</v>
-      </c>
-      <c r="B70" t="s">
-        <v>43</v>
-      </c>
-      <c r="C70" t="s">
-        <v>44</v>
-      </c>
-      <c r="D70" t="s">
-        <v>287</v>
-      </c>
-      <c r="J70" t="s">
-        <v>288</v>
-      </c>
-      <c r="AJ70" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO70" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="71" spans="1:42">
-      <c r="A71" t="s">
-        <v>289</v>
-      </c>
-      <c r="B71" t="s">
-        <v>43</v>
-      </c>
-      <c r="C71" t="s">
-        <v>44</v>
-      </c>
-      <c r="D71" t="s">
-        <v>290</v>
-      </c>
-      <c r="J71" t="s">
-        <v>291</v>
-      </c>
-      <c r="AJ71" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO71" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="72" spans="1:42">
-      <c r="A72" t="s">
-        <v>292</v>
-      </c>
-      <c r="B72" t="s">
-        <v>43</v>
-      </c>
-      <c r="C72" t="s">
-        <v>44</v>
-      </c>
-      <c r="D72" t="s">
-        <v>293</v>
-      </c>
-      <c r="J72" t="s">
-        <v>294</v>
-      </c>
-      <c r="Q72" t="s">
-        <v>295</v>
-      </c>
-      <c r="T72" t="s">
-        <v>296</v>
-      </c>
-      <c r="AJ72" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="73" spans="1:42">
-      <c r="A73" t="s">
-        <v>297</v>
-      </c>
-      <c r="B73" t="s">
-        <v>43</v>
-      </c>
-      <c r="C73" t="s">
-        <v>44</v>
-      </c>
-      <c r="D73" t="s">
-        <v>298</v>
-      </c>
-      <c r="J73" t="s">
-        <v>299</v>
-      </c>
-      <c r="AJ73" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO73" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="74" spans="1:42">
+    <row r="74" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="B74" t="s">
         <v>43</v>
@@ -3568,10 +3578,10 @@
         <v>44</v>
       </c>
       <c r="D74" t="s">
-        <v>301</v>
+        <v>81</v>
       </c>
       <c r="J74" t="s">
-        <v>302</v>
+        <v>82</v>
       </c>
       <c r="AJ74" t="s">
         <v>47</v>
@@ -3580,9 +3590,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="75" spans="1:42">
+    <row r="75" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>303</v>
+        <v>142</v>
       </c>
       <c r="B75" t="s">
         <v>43</v>
@@ -3591,24 +3601,21 @@
         <v>44</v>
       </c>
       <c r="D75" t="s">
-        <v>304</v>
+        <v>143</v>
       </c>
       <c r="J75" t="s">
-        <v>305</v>
-      </c>
-      <c r="S75" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="AJ75" t="s">
         <v>47</v>
       </c>
       <c r="AO75" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="76" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="76" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>306</v>
+        <v>140</v>
       </c>
       <c r="B76" t="s">
         <v>43</v>
@@ -3617,41 +3624,50 @@
         <v>44</v>
       </c>
       <c r="D76" t="s">
-        <v>307</v>
+        <v>369</v>
       </c>
       <c r="J76" t="s">
-        <v>308</v>
+        <v>370</v>
+      </c>
+      <c r="R76" t="s">
+        <v>137</v>
+      </c>
+      <c r="S76" t="s">
+        <v>69</v>
       </c>
       <c r="AJ76" t="s">
         <v>47</v>
       </c>
       <c r="AO76" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="77" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>203</v>
+      </c>
+      <c r="B77" t="s">
+        <v>43</v>
+      </c>
+      <c r="C77" t="s">
+        <v>44</v>
+      </c>
+      <c r="D77" t="s">
+        <v>204</v>
+      </c>
+      <c r="J77" t="s">
+        <v>205</v>
+      </c>
+      <c r="AJ77" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO77" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="77" spans="1:42">
-      <c r="A77" t="s">
-        <v>309</v>
-      </c>
-      <c r="B77" t="s">
-        <v>43</v>
-      </c>
-      <c r="C77" t="s">
-        <v>44</v>
-      </c>
-      <c r="D77" t="s">
-        <v>310</v>
-      </c>
-      <c r="J77" t="s">
-        <v>311</v>
-      </c>
-      <c r="AJ77" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="78" spans="1:42">
+    <row r="78" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>312</v>
+        <v>101</v>
       </c>
       <c r="B78" t="s">
         <v>43</v>
@@ -3660,50 +3676,47 @@
         <v>44</v>
       </c>
       <c r="D78" t="s">
-        <v>313</v>
+        <v>102</v>
       </c>
       <c r="J78" t="s">
-        <v>314</v>
+        <v>103</v>
+      </c>
+      <c r="L78" t="s">
+        <v>104</v>
       </c>
       <c r="AJ78" t="s">
         <v>47</v>
       </c>
       <c r="AO78" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="79" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>256</v>
+      </c>
+      <c r="B79" t="s">
+        <v>43</v>
+      </c>
+      <c r="C79" t="s">
+        <v>44</v>
+      </c>
+      <c r="D79" t="s">
+        <v>257</v>
+      </c>
+      <c r="J79" t="s">
+        <v>258</v>
+      </c>
+      <c r="AJ79" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO79" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="79" spans="1:42">
-      <c r="A79" t="s">
-        <v>315</v>
-      </c>
-      <c r="B79" t="s">
-        <v>43</v>
-      </c>
-      <c r="C79" t="s">
-        <v>44</v>
-      </c>
-      <c r="D79" t="s">
-        <v>316</v>
-      </c>
-      <c r="E79" t="s">
-        <v>317</v>
-      </c>
-      <c r="J79" t="s">
-        <v>318</v>
-      </c>
-      <c r="W79" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ79" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO79" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="80" spans="1:42">
+    <row r="80" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>320</v>
+        <v>337</v>
       </c>
       <c r="B80" t="s">
         <v>43</v>
@@ -3712,10 +3725,13 @@
         <v>44</v>
       </c>
       <c r="D80" t="s">
-        <v>321</v>
+        <v>338</v>
       </c>
       <c r="J80" t="s">
-        <v>322</v>
+        <v>339</v>
+      </c>
+      <c r="S80" t="s">
+        <v>222</v>
       </c>
       <c r="AJ80" t="s">
         <v>47</v>
@@ -3724,9 +3740,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="81" spans="1:42">
+    <row r="81" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B81" t="s">
         <v>43</v>
@@ -3735,27 +3751,21 @@
         <v>44</v>
       </c>
       <c r="D81" t="s">
-        <v>324</v>
-      </c>
-      <c r="F81" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="J81" t="s">
-        <v>326</v>
-      </c>
-      <c r="L81" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="AJ81" t="s">
         <v>47</v>
       </c>
       <c r="AO81" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="82" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="82" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>328</v>
+        <v>88</v>
       </c>
       <c r="B82" t="s">
         <v>43</v>
@@ -3764,73 +3774,73 @@
         <v>44</v>
       </c>
       <c r="D82" t="s">
-        <v>329</v>
+        <v>89</v>
       </c>
       <c r="J82" t="s">
-        <v>330</v>
+        <v>90</v>
+      </c>
+      <c r="R82" t="s">
+        <v>91</v>
       </c>
       <c r="AJ82" t="s">
         <v>47</v>
       </c>
       <c r="AO82" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="83" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>149</v>
+      </c>
+      <c r="B83" t="s">
+        <v>43</v>
+      </c>
+      <c r="C83" t="s">
+        <v>44</v>
+      </c>
+      <c r="D83" t="s">
+        <v>150</v>
+      </c>
+      <c r="J83" t="s">
+        <v>151</v>
+      </c>
+      <c r="L83" t="s">
+        <v>152</v>
+      </c>
+      <c r="AJ83" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO83" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="84" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>117</v>
+      </c>
+      <c r="B84" t="s">
+        <v>43</v>
+      </c>
+      <c r="C84" t="s">
+        <v>44</v>
+      </c>
+      <c r="D84" t="s">
+        <v>118</v>
+      </c>
+      <c r="J84" t="s">
+        <v>119</v>
+      </c>
+      <c r="AJ84" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO84" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="83" spans="1:42">
-      <c r="A83" t="s">
-        <v>331</v>
-      </c>
-      <c r="B83" t="s">
-        <v>43</v>
-      </c>
-      <c r="C83" t="s">
-        <v>44</v>
-      </c>
-      <c r="D83" t="s">
-        <v>332</v>
-      </c>
-      <c r="J83" t="s">
-        <v>333</v>
-      </c>
-      <c r="W83" t="s">
-        <v>162</v>
-      </c>
-      <c r="AJ83" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO83" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="84" spans="1:42">
-      <c r="A84" t="s">
-        <v>334</v>
-      </c>
-      <c r="B84" t="s">
-        <v>43</v>
-      </c>
-      <c r="C84" t="s">
-        <v>44</v>
-      </c>
-      <c r="D84" t="s">
-        <v>335</v>
-      </c>
-      <c r="J84" t="s">
-        <v>336</v>
-      </c>
-      <c r="W84" t="s">
-        <v>91</v>
-      </c>
-      <c r="AJ84" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO84" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="85" spans="1:42">
+    <row r="85" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>337</v>
+        <v>75</v>
       </c>
       <c r="B85" t="s">
         <v>43</v>
@@ -3839,13 +3849,10 @@
         <v>44</v>
       </c>
       <c r="D85" t="s">
-        <v>338</v>
+        <v>76</v>
       </c>
       <c r="J85" t="s">
-        <v>339</v>
-      </c>
-      <c r="S85" t="s">
-        <v>222</v>
+        <v>58</v>
       </c>
       <c r="AJ85" t="s">
         <v>47</v>
@@ -3854,9 +3861,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="86" spans="1:42">
+    <row r="86" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="B86" t="s">
         <v>43</v>
@@ -3865,30 +3872,21 @@
         <v>44</v>
       </c>
       <c r="D86" t="s">
-        <v>340</v>
+        <v>57</v>
       </c>
       <c r="J86" t="s">
-        <v>341</v>
-      </c>
-      <c r="L86" t="s">
-        <v>104</v>
-      </c>
-      <c r="R86" t="s">
-        <v>342</v>
-      </c>
-      <c r="T86" t="s">
-        <v>343</v>
+        <v>58</v>
       </c>
       <c r="AJ86" t="s">
         <v>47</v>
       </c>
       <c r="AO86" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="87" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="87" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>344</v>
+        <v>181</v>
       </c>
       <c r="B87" t="s">
         <v>43</v>
@@ -3897,88 +3895,82 @@
         <v>44</v>
       </c>
       <c r="D87" t="s">
-        <v>345</v>
+        <v>182</v>
       </c>
       <c r="J87" t="s">
-        <v>346</v>
-      </c>
-      <c r="W87" t="s">
+        <v>183</v>
+      </c>
+      <c r="P87" t="s">
+        <v>129</v>
+      </c>
+      <c r="AJ87" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="88" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>389</v>
+      </c>
+      <c r="B88" t="s">
+        <v>43</v>
+      </c>
+      <c r="C88" t="s">
+        <v>44</v>
+      </c>
+      <c r="D88" t="s">
+        <v>390</v>
+      </c>
+      <c r="J88" t="s">
+        <v>391</v>
+      </c>
+      <c r="AJ88" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO88" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="89" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>398</v>
+      </c>
+      <c r="B89" t="s">
+        <v>43</v>
+      </c>
+      <c r="C89" t="s">
+        <v>44</v>
+      </c>
+      <c r="D89" t="s">
+        <v>399</v>
+      </c>
+      <c r="J89" t="s">
+        <v>400</v>
+      </c>
+      <c r="AJ89" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO89" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="90" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>178</v>
+      </c>
+      <c r="B90" t="s">
+        <v>43</v>
+      </c>
+      <c r="C90" t="s">
+        <v>44</v>
+      </c>
+      <c r="D90" t="s">
+        <v>179</v>
+      </c>
+      <c r="J90" t="s">
+        <v>180</v>
+      </c>
+      <c r="W90" t="s">
         <v>91</v>
-      </c>
-      <c r="AJ87" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO87" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="88" spans="1:42">
-      <c r="A88" t="s">
-        <v>222</v>
-      </c>
-      <c r="B88" t="s">
-        <v>43</v>
-      </c>
-      <c r="C88" t="s">
-        <v>44</v>
-      </c>
-      <c r="D88" t="s">
-        <v>348</v>
-      </c>
-      <c r="J88" t="s">
-        <v>349</v>
-      </c>
-      <c r="S88" t="s">
-        <v>292</v>
-      </c>
-      <c r="T88" t="s">
-        <v>350</v>
-      </c>
-      <c r="AJ88" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="89" spans="1:42">
-      <c r="A89" t="s">
-        <v>74</v>
-      </c>
-      <c r="B89" t="s">
-        <v>43</v>
-      </c>
-      <c r="C89" t="s">
-        <v>44</v>
-      </c>
-      <c r="D89" t="s">
-        <v>351</v>
-      </c>
-      <c r="J89" t="s">
-        <v>352</v>
-      </c>
-      <c r="P89" t="s">
-        <v>71</v>
-      </c>
-      <c r="AJ89" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO89" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="90" spans="1:42">
-      <c r="A90" t="s">
-        <v>353</v>
-      </c>
-      <c r="B90" t="s">
-        <v>43</v>
-      </c>
-      <c r="C90" t="s">
-        <v>44</v>
-      </c>
-      <c r="D90" t="s">
-        <v>354</v>
-      </c>
-      <c r="J90" t="s">
-        <v>355</v>
       </c>
       <c r="AJ90" t="s">
         <v>47</v>
@@ -3987,9 +3979,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="91" spans="1:42">
+    <row r="91" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>356</v>
+        <v>300</v>
       </c>
       <c r="B91" t="s">
         <v>43</v>
@@ -3998,10 +3990,10 @@
         <v>44</v>
       </c>
       <c r="D91" t="s">
-        <v>357</v>
+        <v>301</v>
       </c>
       <c r="J91" t="s">
-        <v>358</v>
+        <v>302</v>
       </c>
       <c r="AJ91" t="s">
         <v>47</v>
@@ -4010,9 +4002,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="92" spans="1:42">
+    <row r="92" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>359</v>
+        <v>120</v>
       </c>
       <c r="B92" t="s">
         <v>43</v>
@@ -4021,24 +4013,24 @@
         <v>44</v>
       </c>
       <c r="D92" t="s">
-        <v>360</v>
-      </c>
-      <c r="G92" t="s">
-        <v>361</v>
+        <v>121</v>
       </c>
       <c r="J92" t="s">
-        <v>362</v>
-      </c>
-      <c r="S92" t="s">
-        <v>292</v>
+        <v>122</v>
+      </c>
+      <c r="W92" t="s">
+        <v>91</v>
       </c>
       <c r="AJ92" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="93" spans="1:42">
+      <c r="AO92" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="93" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>162</v>
+        <v>277</v>
       </c>
       <c r="B93" t="s">
         <v>43</v>
@@ -4047,30 +4039,21 @@
         <v>44</v>
       </c>
       <c r="D93" t="s">
-        <v>363</v>
+        <v>278</v>
       </c>
       <c r="J93" t="s">
-        <v>364</v>
-      </c>
-      <c r="L93" t="s">
-        <v>104</v>
-      </c>
-      <c r="R93" t="s">
-        <v>59</v>
-      </c>
-      <c r="X93" t="s">
-        <v>365</v>
+        <v>279</v>
       </c>
       <c r="AJ93" t="s">
         <v>47</v>
       </c>
       <c r="AO93" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="94" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="94" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>366</v>
+        <v>312</v>
       </c>
       <c r="B94" t="s">
         <v>43</v>
@@ -4079,24 +4062,21 @@
         <v>44</v>
       </c>
       <c r="D94" t="s">
-        <v>367</v>
+        <v>313</v>
       </c>
       <c r="J94" t="s">
-        <v>368</v>
-      </c>
-      <c r="W94" t="s">
-        <v>162</v>
+        <v>314</v>
       </c>
       <c r="AJ94" t="s">
         <v>47</v>
       </c>
       <c r="AO94" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="95" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="95" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>140</v>
+        <v>52</v>
       </c>
       <c r="B95" t="s">
         <v>43</v>
@@ -4105,27 +4085,21 @@
         <v>44</v>
       </c>
       <c r="D95" t="s">
-        <v>369</v>
+        <v>53</v>
       </c>
       <c r="J95" t="s">
-        <v>370</v>
-      </c>
-      <c r="R95" t="s">
-        <v>137</v>
-      </c>
-      <c r="S95" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="AJ95" t="s">
         <v>47</v>
       </c>
       <c r="AO95" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="96" spans="1:42">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="96" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>295</v>
+        <v>265</v>
       </c>
       <c r="B96" t="s">
         <v>43</v>
@@ -4134,24 +4108,21 @@
         <v>44</v>
       </c>
       <c r="D96" t="s">
-        <v>371</v>
+        <v>266</v>
       </c>
       <c r="J96" t="s">
-        <v>372</v>
-      </c>
-      <c r="P96" t="s">
-        <v>292</v>
+        <v>267</v>
       </c>
       <c r="AJ96" t="s">
         <v>47</v>
       </c>
       <c r="AO96" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="97" spans="1:42">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="97" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>373</v>
+        <v>200</v>
       </c>
       <c r="B97" t="s">
         <v>43</v>
@@ -4160,10 +4131,10 @@
         <v>44</v>
       </c>
       <c r="D97" t="s">
-        <v>374</v>
+        <v>201</v>
       </c>
       <c r="J97" t="s">
-        <v>375</v>
+        <v>202</v>
       </c>
       <c r="AJ97" t="s">
         <v>47</v>
@@ -4172,9 +4143,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="98" spans="1:42">
+    <row r="98" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>376</v>
+        <v>174</v>
       </c>
       <c r="B98" t="s">
         <v>43</v>
@@ -4183,44 +4154,53 @@
         <v>44</v>
       </c>
       <c r="D98" t="s">
-        <v>377</v>
+        <v>413</v>
       </c>
       <c r="J98" t="s">
-        <v>378</v>
+        <v>414</v>
+      </c>
+      <c r="R98" t="s">
+        <v>171</v>
       </c>
       <c r="AJ98" t="s">
         <v>47</v>
       </c>
       <c r="AO98" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="99" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>171</v>
+      </c>
+      <c r="B99" t="s">
+        <v>43</v>
+      </c>
+      <c r="C99" t="s">
+        <v>44</v>
+      </c>
+      <c r="D99" t="s">
+        <v>172</v>
+      </c>
+      <c r="J99" t="s">
+        <v>173</v>
+      </c>
+      <c r="R99" t="s">
+        <v>174</v>
+      </c>
+      <c r="W99" t="s">
+        <v>91</v>
+      </c>
+      <c r="AJ99" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO99" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="99" spans="1:42">
-      <c r="A99" t="s">
-        <v>379</v>
-      </c>
-      <c r="B99" t="s">
-        <v>43</v>
-      </c>
-      <c r="C99" t="s">
-        <v>44</v>
-      </c>
-      <c r="D99" t="s">
-        <v>380</v>
-      </c>
-      <c r="J99" t="s">
-        <v>381</v>
-      </c>
-      <c r="AJ99" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO99" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="100" spans="1:42">
+    <row r="100" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>383</v>
+        <v>268</v>
       </c>
       <c r="B100" t="s">
         <v>43</v>
@@ -4229,21 +4209,21 @@
         <v>44</v>
       </c>
       <c r="D100" t="s">
-        <v>384</v>
+        <v>269</v>
       </c>
       <c r="J100" t="s">
-        <v>385</v>
+        <v>270</v>
+      </c>
+      <c r="S100" t="s">
+        <v>69</v>
       </c>
       <c r="AJ100" t="s">
         <v>47</v>
       </c>
-      <c r="AO100" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="101" spans="1:42">
+    </row>
+    <row r="101" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>386</v>
+        <v>175</v>
       </c>
       <c r="B101" t="s">
         <v>43</v>
@@ -4252,10 +4232,10 @@
         <v>44</v>
       </c>
       <c r="D101" t="s">
-        <v>387</v>
+        <v>176</v>
       </c>
       <c r="J101" t="s">
-        <v>388</v>
+        <v>177</v>
       </c>
       <c r="AJ101" t="s">
         <v>47</v>
@@ -4264,9 +4244,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="102" spans="1:42">
+    <row r="102" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>389</v>
+        <v>111</v>
       </c>
       <c r="B102" t="s">
         <v>43</v>
@@ -4275,10 +4255,10 @@
         <v>44</v>
       </c>
       <c r="D102" t="s">
-        <v>390</v>
+        <v>112</v>
       </c>
       <c r="J102" t="s">
-        <v>391</v>
+        <v>113</v>
       </c>
       <c r="AJ102" t="s">
         <v>47</v>
@@ -4287,9 +4267,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="103" spans="1:42">
+    <row r="103" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>392</v>
+        <v>344</v>
       </c>
       <c r="B103" t="s">
         <v>43</v>
@@ -4298,21 +4278,24 @@
         <v>44</v>
       </c>
       <c r="D103" t="s">
-        <v>393</v>
+        <v>345</v>
       </c>
       <c r="J103" t="s">
-        <v>394</v>
+        <v>346</v>
+      </c>
+      <c r="W103" t="s">
+        <v>91</v>
       </c>
       <c r="AJ103" t="s">
         <v>47</v>
       </c>
       <c r="AO103" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="104" spans="1:42">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="104" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>395</v>
+        <v>49</v>
       </c>
       <c r="B104" t="s">
         <v>43</v>
@@ -4321,10 +4304,10 @@
         <v>44</v>
       </c>
       <c r="D104" t="s">
-        <v>396</v>
+        <v>50</v>
       </c>
       <c r="J104" t="s">
-        <v>397</v>
+        <v>51</v>
       </c>
       <c r="AJ104" t="s">
         <v>47</v>
@@ -4333,9 +4316,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="105" spans="1:42">
+    <row r="105" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>398</v>
+        <v>123</v>
       </c>
       <c r="B105" t="s">
         <v>43</v>
@@ -4344,67 +4327,67 @@
         <v>44</v>
       </c>
       <c r="D105" t="s">
-        <v>399</v>
+        <v>124</v>
       </c>
       <c r="J105" t="s">
-        <v>400</v>
+        <v>125</v>
       </c>
       <c r="AJ105" t="s">
         <v>47</v>
       </c>
       <c r="AO105" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="106" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>404</v>
+      </c>
+      <c r="B106" t="s">
+        <v>43</v>
+      </c>
+      <c r="C106" t="s">
+        <v>44</v>
+      </c>
+      <c r="D106" t="s">
+        <v>405</v>
+      </c>
+      <c r="J106" t="s">
+        <v>406</v>
+      </c>
+      <c r="AJ106" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO106" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="106" spans="1:42">
-      <c r="A106" t="s">
-        <v>401</v>
-      </c>
-      <c r="B106" t="s">
-        <v>43</v>
-      </c>
-      <c r="C106" t="s">
-        <v>44</v>
-      </c>
-      <c r="D106" t="s">
-        <v>402</v>
-      </c>
-      <c r="J106" t="s">
-        <v>403</v>
-      </c>
-      <c r="AJ106" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO106" t="s">
+    <row r="107" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>373</v>
+      </c>
+      <c r="B107" t="s">
+        <v>43</v>
+      </c>
+      <c r="C107" t="s">
+        <v>44</v>
+      </c>
+      <c r="D107" t="s">
+        <v>374</v>
+      </c>
+      <c r="J107" t="s">
+        <v>375</v>
+      </c>
+      <c r="AJ107" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO107" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="107" spans="1:42">
-      <c r="A107" t="s">
-        <v>404</v>
-      </c>
-      <c r="B107" t="s">
-        <v>43</v>
-      </c>
-      <c r="C107" t="s">
-        <v>44</v>
-      </c>
-      <c r="D107" t="s">
-        <v>405</v>
-      </c>
-      <c r="J107" t="s">
-        <v>406</v>
-      </c>
-      <c r="AJ107" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO107" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="108" spans="1:42">
+    <row r="108" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>407</v>
+        <v>328</v>
       </c>
       <c r="B108" t="s">
         <v>43</v>
@@ -4413,10 +4396,10 @@
         <v>44</v>
       </c>
       <c r="D108" t="s">
-        <v>408</v>
+        <v>329</v>
       </c>
       <c r="J108" t="s">
-        <v>409</v>
+        <v>330</v>
       </c>
       <c r="AJ108" t="s">
         <v>47</v>
@@ -4425,167 +4408,186 @@
         <v>48</v>
       </c>
     </row>
-    <row r="109" spans="1:42">
+    <row r="109" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>69</v>
+      </c>
+      <c r="B109" t="s">
+        <v>43</v>
+      </c>
+      <c r="C109" t="s">
+        <v>44</v>
+      </c>
+      <c r="D109" t="s">
+        <v>340</v>
+      </c>
+      <c r="J109" t="s">
+        <v>341</v>
+      </c>
+      <c r="L109" t="s">
+        <v>104</v>
+      </c>
+      <c r="R109" t="s">
+        <v>342</v>
+      </c>
+      <c r="T109" t="s">
+        <v>343</v>
+      </c>
+      <c r="AJ109" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO109" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="110" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>188</v>
+      </c>
+      <c r="B110" t="s">
+        <v>43</v>
+      </c>
+      <c r="C110" t="s">
+        <v>44</v>
+      </c>
+      <c r="D110" t="s">
+        <v>189</v>
+      </c>
+      <c r="E110" t="s">
+        <v>190</v>
+      </c>
+      <c r="J110" t="s">
+        <v>191</v>
+      </c>
+      <c r="R110" t="s">
+        <v>69</v>
+      </c>
+      <c r="AJ110" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="111" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>280</v>
+      </c>
+      <c r="B111" t="s">
+        <v>43</v>
+      </c>
+      <c r="C111" t="s">
+        <v>44</v>
+      </c>
+      <c r="D111" t="s">
+        <v>281</v>
+      </c>
+      <c r="J111" t="s">
+        <v>282</v>
+      </c>
+      <c r="AJ111" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO111" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="112" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>415</v>
+      </c>
+      <c r="B112" t="s">
+        <v>43</v>
+      </c>
+      <c r="C112" t="s">
+        <v>44</v>
+      </c>
+      <c r="D112" t="s">
+        <v>416</v>
+      </c>
+      <c r="J112" t="s">
+        <v>417</v>
+      </c>
+      <c r="AI112" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="113" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>129</v>
+      </c>
+      <c r="B113" t="s">
+        <v>43</v>
+      </c>
+      <c r="C113" t="s">
+        <v>44</v>
+      </c>
+      <c r="D113" t="s">
+        <v>212</v>
+      </c>
+      <c r="J113" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>181</v>
+      </c>
+      <c r="T113" t="s">
+        <v>214</v>
+      </c>
+      <c r="AJ113" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="114" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>331</v>
+      </c>
+      <c r="B114" t="s">
+        <v>43</v>
+      </c>
+      <c r="C114" t="s">
+        <v>44</v>
+      </c>
+      <c r="D114" t="s">
+        <v>332</v>
+      </c>
+      <c r="J114" t="s">
+        <v>333</v>
+      </c>
+      <c r="W114" t="s">
+        <v>162</v>
+      </c>
+      <c r="AJ114" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO114" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="115" spans="1:41" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>410</v>
       </c>
-      <c r="B109" t="s">
-        <v>43</v>
-      </c>
-      <c r="C109" t="s">
-        <v>44</v>
-      </c>
-      <c r="D109" t="s">
+      <c r="B115" t="s">
+        <v>43</v>
+      </c>
+      <c r="C115" t="s">
+        <v>44</v>
+      </c>
+      <c r="D115" t="s">
         <v>411</v>
       </c>
-      <c r="J109" t="s">
+      <c r="J115" t="s">
         <v>412</v>
       </c>
-      <c r="AJ109" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO109" t="s">
+      <c r="AJ115" t="s">
+        <v>47</v>
+      </c>
+      <c r="AO115" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="110" spans="1:42">
-      <c r="A110" t="s">
-        <v>174</v>
-      </c>
-      <c r="B110" t="s">
-        <v>43</v>
-      </c>
-      <c r="C110" t="s">
-        <v>44</v>
-      </c>
-      <c r="D110" t="s">
-        <v>413</v>
-      </c>
-      <c r="J110" t="s">
-        <v>414</v>
-      </c>
-      <c r="R110" t="s">
-        <v>171</v>
-      </c>
-      <c r="AJ110" t="s">
-        <v>47</v>
-      </c>
-      <c r="AO110" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="111" spans="1:42">
-      <c r="A111" t="s">
-        <v>415</v>
-      </c>
-      <c r="B111" t="s">
-        <v>43</v>
-      </c>
-      <c r="C111" t="s">
-        <v>44</v>
-      </c>
-      <c r="D111" t="s">
-        <v>416</v>
-      </c>
-      <c r="J111" t="s">
-        <v>417</v>
-      </c>
-      <c r="AI111" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="112" spans="1:42">
-      <c r="A112" t="s">
-        <v>419</v>
-      </c>
-      <c r="B112" t="s">
-        <v>43</v>
-      </c>
-      <c r="C112" t="s">
-        <v>44</v>
-      </c>
-      <c r="D112" t="s">
-        <v>420</v>
-      </c>
-      <c r="J112" t="s">
-        <v>421</v>
-      </c>
-      <c r="AO112" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="113" spans="1:42">
-      <c r="A113" t="s">
-        <v>423</v>
-      </c>
-      <c r="B113" t="s">
-        <v>43</v>
-      </c>
-      <c r="C113" t="s">
-        <v>44</v>
-      </c>
-      <c r="D113" t="s">
-        <v>424</v>
-      </c>
-      <c r="J113" t="s">
-        <v>425</v>
-      </c>
-      <c r="AO113" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="114" spans="1:42">
-      <c r="A114" t="s">
-        <v>426</v>
-      </c>
-      <c r="B114" t="s">
-        <v>43</v>
-      </c>
-      <c r="C114" t="s">
-        <v>44</v>
-      </c>
-      <c r="D114" t="s">
-        <v>427</v>
-      </c>
-      <c r="J114" t="s">
-        <v>428</v>
-      </c>
-      <c r="AO114" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="115" spans="1:42">
-      <c r="A115" t="s">
-        <v>429</v>
-      </c>
-      <c r="B115" t="s">
-        <v>43</v>
-      </c>
-      <c r="C115" t="s">
-        <v>44</v>
-      </c>
-      <c r="D115" t="s">
-        <v>430</v>
-      </c>
-      <c r="J115" t="s">
-        <v>431</v>
-      </c>
-      <c r="AO115" t="s">
-        <v>422</v>
-      </c>
-    </row>
   </sheetData>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AP115">
+    <sortCondition ref="D2:D115"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>